<commit_message>
Update assets/档案体系总览-脱敏版.xlsx (renumber C01-C21)
</commit_message>
<xml_diff>
--- a/assets/档案体系总览-脱敏版.xlsx
+++ b/assets/档案体系总览-脱敏版.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="档案体系总览（脱敏版）" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类总览（C01-C21）" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,58 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="微软雅黑"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="微软雅黑"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="微软雅黑"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="微软雅黑"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="微软雅黑"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEF2F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCE6F1"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,17 +84,43 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C9D3E0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C9D3E0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9D3E0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C9D3E0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -419,549 +487,568 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>翟靖昊 · 学校文件分类整理体系（脱敏版）</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr"/>
-      <c r="C1" t="inlineStr"/>
-      <c r="D1" t="inlineStr"/>
-      <c r="E1" t="inlineStr"/>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>说明：本表仅含分类体系元数据，不含任何学生个人信息；已剔除软件工具与游戏娱乐类（C20）。</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>翟靖昊 · 学校文件分类整理体系（脱敏版 · 重编号）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>说明：本表仅含分类体系元数据，不含任何学生个人信息；已删除“软件工具与游戏娱乐”，分类重编号为 C01–C21 连续。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>分类编号</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>分类名称</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>用途说明</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>文件数</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>总大小(MB)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>C01</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>学生花名册与基本信息</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>各班学生名单、花名册、录取/学籍信息、新生信息导入表、学生银行卡等基础信息表</t>
         </is>
       </c>
-      <c r="D4" s="1" t="n">
+      <c r="D4" s="4" t="n">
         <v>76</v>
       </c>
-      <c r="E4" s="1" t="n">
+      <c r="E4" s="4" t="n">
         <v>31.4</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>C02</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>成绩与排名</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>期末成绩、平均成绩、班级/专业排名、成绩汇总表</t>
         </is>
       </c>
-      <c r="D5" s="1" t="n">
+      <c r="D5" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="E5" s="1" t="n">
+      <c r="E5" s="5" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>C03</t>
         </is>
       </c>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>综合素质测评</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>综合素质测评表、每月综合成绩与扣分明细、综合素质评价排名</t>
         </is>
       </c>
-      <c r="D6" s="1" t="n">
+      <c r="D6" s="4" t="n">
         <v>54</v>
       </c>
-      <c r="E6" s="1" t="n">
+      <c r="E6" s="4" t="n">
         <v>25.8</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>C04</t>
         </is>
       </c>
-      <c r="B7" s="1" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>考试报名与考证（英语、日语、电工等）</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>英语A级/B级、英语四级、日语四级报名名单、报名表、报名照片，电工四级鉴定及报考材料</t>
         </is>
       </c>
-      <c r="D7" s="1" t="n">
+      <c r="D7" s="5" t="n">
         <v>354</v>
       </c>
-      <c r="E7" s="1" t="n">
+      <c r="E7" s="5" t="n">
         <v>45.8</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>C05</t>
         </is>
       </c>
-      <c r="B8" s="1" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>奖助学金与困难补助</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>国家励志奖学金、国家助学金、特困补助、助学贷款、相关导入模板与备查汇总表</t>
         </is>
       </c>
-      <c r="D8" s="1" t="n">
+      <c r="D8" s="4" t="n">
         <v>21</v>
       </c>
-      <c r="E8" s="1" t="n">
+      <c r="E8" s="4" t="n">
         <v>1.6</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>C06</t>
         </is>
       </c>
-      <c r="B9" s="1" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>家庭经济信息（六类、非六类）</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>六类/非六类家庭经济困难学生信息录入表</t>
         </is>
       </c>
-      <c r="D9" s="1" t="n">
+      <c r="D9" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="E9" s="1" t="n">
+      <c r="E9" s="5" t="n">
         <v>3.5</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>C07</t>
         </is>
       </c>
-      <c r="B10" s="1" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>党团建设材料</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>团员名单/团费/团员评议/推优、入党积极分子与党员发展全流程材料、公示、政审、党纪学习</t>
         </is>
       </c>
-      <c r="D10" s="1" t="n">
+      <c r="D10" s="4" t="n">
         <v>91</v>
       </c>
-      <c r="E10" s="1" t="n">
+      <c r="E10" s="4" t="n">
         <v>210.8</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>C08</t>
         </is>
       </c>
-      <c r="B11" s="1" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>荣誉证书与评优评先</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>三好学生、优秀干部、优秀团员、优秀毕业生审批表/登记表、个人荣誉证书照片</t>
         </is>
       </c>
-      <c r="D11" s="1" t="n">
+      <c r="D11" s="5" t="n">
         <v>43</v>
       </c>
-      <c r="E11" s="1" t="n">
+      <c r="E11" s="5" t="n">
         <v>32</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>C09</t>
         </is>
       </c>
-      <c r="B12" s="1" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>学籍证明与火车票优惠</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>学生学籍证明、团体学籍名册、高铁学生票购票信息表</t>
         </is>
       </c>
-      <c r="D12" s="1" t="n">
+      <c r="D12" s="4" t="n">
         <v>31</v>
       </c>
-      <c r="E12" s="1" t="n">
+      <c r="E12" s="4" t="n">
         <v>3.6</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>C10</t>
         </is>
       </c>
-      <c r="B13" s="1" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>班级日常管理</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>班会记录与总结、放假留校/离校名单、值岗值日、献血名单、技能特长、评教、考勤照片</t>
         </is>
       </c>
-      <c r="D13" s="1" t="n">
+      <c r="D13" s="5" t="n">
         <v>59</v>
       </c>
-      <c r="E13" s="1" t="n">
+      <c r="E13" s="5" t="n">
         <v>49.4</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>C11</t>
         </is>
       </c>
-      <c r="B14" s="1" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>课程教学与学习资料</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>课表、课程标准与考核方案、课程安排、复习题/试题/答案、补考与考场安排、讲稿、教学PPT</t>
         </is>
       </c>
-      <c r="D14" s="1" t="n">
+      <c r="D14" s="4" t="n">
         <v>55</v>
       </c>
-      <c r="E14" s="1" t="n">
+      <c r="E14" s="4" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>C12</t>
         </is>
       </c>
-      <c r="B15" s="1" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>就业与职业规划</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>职业生涯规划书/PPT、职业规划大赛通知与材料、求职简历、就业展示PPT</t>
         </is>
       </c>
-      <c r="D15" s="1" t="n">
+      <c r="D15" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="E15" s="1" t="n">
+      <c r="E15" s="5" t="n">
         <v>68.90000000000001</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>C13</t>
         </is>
       </c>
-      <c r="B16" s="1" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>毕业论文与毕业设计</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>电气专业毕业设计论文（PLC、电梯、交通灯、喷泉等）及论文模板</t>
         </is>
       </c>
-      <c r="D16" s="1" t="n">
+      <c r="D16" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="E16" s="1" t="n">
+      <c r="E16" s="4" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>C14</t>
         </is>
       </c>
-      <c r="B17" s="1" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>学生证件照与电子照片</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>按身份证号/班级存放的学生电子证件照（3+2、二班、四班、牛马新作、照片压缩包等）</t>
         </is>
       </c>
-      <c r="D17" s="1" t="n">
+      <c r="D17" s="5" t="n">
         <v>932</v>
       </c>
-      <c r="E17" s="1" t="n">
+      <c r="E17" s="5" t="n">
         <v>2212.7</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>C15</t>
         </is>
       </c>
-      <c r="B18" s="1" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>活动照片与班级照片</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>网课照片、班级集体照片/视频等</t>
         </is>
       </c>
-      <c r="D18" s="1" t="n">
+      <c r="D18" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="E18" s="1" t="n">
+      <c r="E18" s="4" t="n">
         <v>33.6</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>C16</t>
         </is>
       </c>
-      <c r="B19" s="1" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>安全与主题教育活动</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>国家安全、防溺水、消防、反诈、宪法、征文等主题教育与班会材料</t>
         </is>
       </c>
-      <c r="D19" s="1" t="n">
+      <c r="D19" s="5" t="n">
         <v>21</v>
       </c>
-      <c r="E19" s="1" t="n">
+      <c r="E19" s="5" t="n">
         <v>53.4</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>C17</t>
         </is>
       </c>
-      <c r="B20" s="1" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>生活事务与通知（医保、献血等）</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>医保参保须知与政策、城乡居民批量采集、献血前后指导等</t>
         </is>
       </c>
-      <c r="D20" s="1" t="n">
+      <c r="D20" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="E20" s="1" t="n">
+      <c r="E20" s="4" t="n">
         <v>4.7</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>C18</t>
         </is>
       </c>
-      <c r="B21" s="1" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>工作总结与述职报告</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>辅导员/教师学期工作总结、述职报告、公众号宣传稿</t>
         </is>
       </c>
-      <c r="D21" s="1" t="n">
+      <c r="D21" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="E21" s="1" t="n">
+      <c r="E21" s="5" t="n">
         <v>78.40000000000001</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="inlineStr">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>C19</t>
         </is>
       </c>
-      <c r="B22" s="1" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>创新创业项目</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>学生创业计划书（环保水瓶、茶舍等）</t>
         </is>
       </c>
-      <c r="D22" s="1" t="n">
+      <c r="D22" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E22" s="1" t="n">
+      <c r="E22" s="4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="inlineStr">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>C20</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>学生个人材料与作业</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>学生个人专属材料、课程作业与个人文稿</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>C21</t>
         </is>
       </c>
-      <c r="B23" s="1" t="inlineStr">
-        <is>
-          <t>学生个人材料与作业</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>学生个人专属材料、课程作业与个人文稿</t>
-        </is>
-      </c>
-      <c r="D23" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="E23" s="1" t="n">
-        <v>1.3</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>C22</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>其他未分类杂项</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>空文档、临时文件、录音、来源不明的文件，建议人工核对</t>
         </is>
       </c>
-      <c r="D24" s="1" t="n">
+      <c r="D24" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="E24" s="1" t="n">
+      <c r="E24" s="4" t="n">
         <v>7.1</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>合计</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>21 类</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>1904</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>2892</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>